<commit_message>
feat(pastry-shop-guide-en): entregables definitivos tras la revisión (guía 113 págs., bonus 39, plan, 8 xlsx con gate)
Via: Claude Code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/how-to-open-a-pastry-shop/3-year-financial-plan.xlsx
+++ b/astro-site/public/dl/how-to-open-a-pastry-shop/3-year-financial-plan.xlsx
@@ -2377,7 +2377,7 @@
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>How far you can fall below plan before you start losing money.</t>
+          <t>Minimum margin of the plan over break-even, measured over break-even (the drop in sales it absorbs is smaller: 1 − 1/(1 + this %)).</t>
         </is>
       </c>
     </row>
@@ -4838,7 +4838,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>How far you can fall below plan before you can't pay the fixed costs and the loan payment. The minimum required is in "0. Assumptions".</t>
+          <t>How far the plan sits above CASH break-even. The drop in sales it can absorb is smaller: 1 − 1/(1 + this %), about 18.6% in the case. The minimum required is in "0. Assumptions".</t>
         </is>
       </c>
     </row>

</xml_diff>